<commit_message>
[B1] Drop duplicate Date Applied column; realign tracker metadata
- Remove the duplicate "Date Applied" column (column E); keep the single
  Date Applied column.
- Rebuild Status/Job Type dropdowns and status color-coding onto the correct
  columns, fixing a pre-existing off-by-one where they partly landed on the
  date columns.
- Repair Dashboard COUNTIF/COUNTIFS formulas after the column shift, and fix
  references that pointed at the wrong columns (status counts/ratios were
  reading date columns).
- Tighten the title-banner merge to the data width (A1:W1).
- Point the process-opportunities skill at the actual "Sourced From (w/link)"
  column instead of a generic "Job URL".

Refs #24

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/job_tracker_template.xlsx
+++ b/templates/job_tracker_template.xlsx
@@ -614,25 +614,19 @@
     <author>Marc Alexander</author>
   </authors>
   <commentList>
-    <comment ref="E3" authorId="0" shapeId="0">
-      <text>
-        <t>Marc Alexander:
-I only apply to ~90% of the opportunities I log here.  Sometimes, after further review, it's not a good match and not worth the application.</t>
-      </text>
-    </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
+    <comment ref="I3" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Marc Alexander:
 Available in Linkedin (might require Premium).  I try to apply 1st day the opportunity posts and be in the 1st 100 applications. </t>
       </text>
     </comment>
-    <comment ref="N3" authorId="0" shapeId="0">
+    <comment ref="M3" authorId="0" shapeId="0">
       <text>
         <t>Marc Alexander:
 Date this applications effectively closed.  This will help determine avg response time for applications supmitted.  It's a valuable data point, but it takes some dlilgence to create good data.</t>
       </text>
     </comment>
-    <comment ref="S3" authorId="0" shapeId="0">
+    <comment ref="R3" authorId="0" shapeId="0">
       <text>
         <t>Marc Alexander:
 If you indicated a salary expectation, log it here so you can recall during a screening call (it happens frequently)</t>
@@ -868,11 +862,11 @@
     </row>
     <row r="6" ht="19.5" customHeight="1" s="42">
       <c r="B6" s="46">
-        <f>COUNTIF('📋 Applications'!E4:E715,"&gt;1")</f>
+        <f>COUNTIF('📋 Applications'!N4:N715,"&gt;1")</f>
         <v/>
       </c>
       <c r="E6" s="47">
-        <f>COUNTIF('📋 Applications'!E4:E715,"In Progress")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"In Progress")</f>
         <v/>
       </c>
     </row>
@@ -891,11 +885,11 @@
     </row>
     <row r="9" ht="19.5" customHeight="1" s="42">
       <c r="B9" s="53">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Offer")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Offer")</f>
         <v/>
       </c>
       <c r="E9" s="44">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Rejected")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Rejected")</f>
         <v/>
       </c>
     </row>
@@ -920,7 +914,7 @@
         </is>
       </c>
       <c r="C13" s="3">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Applied")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Applied")</f>
         <v/>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -941,7 +935,7 @@
         </is>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Phone Screen")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Phone Screen")</f>
         <v/>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -950,7 +944,7 @@
         </is>
       </c>
       <c r="F14" s="3">
-        <f>COUNTIFS('📋 Applications'!E4:E715,"&gt;="&amp;TODAY()-7,'📋 Applications'!E4:E715,"&lt;="&amp;TODAY())</f>
+        <f>COUNTIFS('📋 Applications'!N4:N715,"&gt;="&amp;TODAY()-7,'📋 Applications'!N4:N715,"&lt;="&amp;TODAY())</f>
         <v/>
       </c>
     </row>
@@ -961,7 +955,7 @@
         </is>
       </c>
       <c r="C15" s="3">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Interview")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Interview")</f>
         <v/>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -970,7 +964,7 @@
         </is>
       </c>
       <c r="F15" s="6">
-        <f>COUNTIFS('📋 Applications'!E4:E715,"&gt;="&amp;TODAY()-30,'📋 Applications'!E4:E715,"&lt;="&amp;TODAY())</f>
+        <f>COUNTIFS('📋 Applications'!N4:N715,"&gt;="&amp;TODAY()-30,'📋 Applications'!N4:N715,"&lt;="&amp;TODAY())</f>
         <v/>
       </c>
     </row>
@@ -981,7 +975,7 @@
         </is>
       </c>
       <c r="C16" s="6">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Final Round")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Final Round")</f>
         <v/>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -998,7 +992,7 @@
         </is>
       </c>
       <c r="C17" s="3">
-        <f>COUNTIF('📋 Applications'!M4:M715,"In Progress")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"In Progress")</f>
         <v/>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1015,7 +1009,7 @@
         </is>
       </c>
       <c r="C18" s="6">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Offer")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Offer")</f>
         <v/>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1024,7 +1018,7 @@
         </is>
       </c>
       <c r="F18" s="9">
-        <f>IFERROR(COUNTIFS('📋 Applications'!N4:N715,"Interview")/COUNTA('📋 Applications'!C4:C715),0)</f>
+        <f>IFERROR(COUNTIFS('📋 Applications'!L4:L715,"Interview")/COUNTA('📋 Applications'!C4:C715),0)</f>
         <v/>
       </c>
     </row>
@@ -1035,7 +1029,7 @@
         </is>
       </c>
       <c r="C19" s="3">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Rejected")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Rejected")</f>
         <v/>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1044,7 +1038,7 @@
         </is>
       </c>
       <c r="F19" s="8">
-        <f>IFERROR(COUNTIF('📋 Applications'!N4:N715,"Offer")/COUNTA('📋 Applications'!C4:C715),0)</f>
+        <f>IFERROR(COUNTIF('📋 Applications'!L4:L715,"Offer")/COUNTA('📋 Applications'!C4:C715),0)</f>
         <v/>
       </c>
     </row>
@@ -1055,7 +1049,7 @@
         </is>
       </c>
       <c r="C20" s="6">
-        <f>COUNTIF('📋 Applications'!M4:M715,"Withdrawn")</f>
+        <f>COUNTIF('📋 Applications'!L4:L715,"Withdrawn")</f>
         <v/>
       </c>
     </row>
@@ -1122,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="42" min="1" max="1"/>
@@ -1178,18 +1172,17 @@
       <c r="U2" s="40" t="n"/>
       <c r="V2" s="40" t="n"/>
       <c r="W2" s="40" t="n"/>
-      <c r="X2" s="40" t="n"/>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>P1 Score</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>P1 Score</t>
+          <t>P2 Score</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
-        <is>
-          <t>P2 Score</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
         <is>
           <t>P3 Score</t>
         </is>
@@ -1216,102 +1209,97 @@
           <t>Date Found</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>Role / Title</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Re/Post</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Re/Post Date</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t># Applied</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>Job Type</t>
+        </is>
+      </c>
+      <c r="K3" s="60" t="inlineStr">
+        <is>
+          <t>Resume Score</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>Date Closed</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
         <is>
           <t>Date Applied</t>
         </is>
       </c>
-      <c r="F3" s="26" t="inlineStr">
-        <is>
-          <t>Role / Title</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>Re/Post</t>
-        </is>
-      </c>
-      <c r="I3" s="10" t="inlineStr">
-        <is>
-          <t>Re/Post Date</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t># Applied</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>Job Type</t>
-        </is>
-      </c>
-      <c r="L3" s="60" t="inlineStr">
-        <is>
-          <t>Resume Score</t>
-        </is>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>Date Closed</t>
-        </is>
-      </c>
       <c r="O3" s="10" t="inlineStr">
         <is>
-          <t>Date Applied</t>
+          <t>Salary (Min)</t>
         </is>
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
-          <t>Salary (Min)</t>
+          <t>Salary (Max)</t>
         </is>
       </c>
       <c r="Q3" s="10" t="inlineStr">
         <is>
-          <t>Salary (Max)</t>
+          <t>Sourced From (w/link)</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Sourced From (w/link)</t>
+          <t>Expected Salary</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
         <is>
-          <t>Expected Salary</t>
+          <t>Contact Name</t>
         </is>
       </c>
       <c r="T3" s="10" t="inlineStr">
         <is>
-          <t>Contact Name</t>
+          <t>Contact Email</t>
         </is>
       </c>
       <c r="U3" s="10" t="inlineStr">
         <is>
-          <t>Contact Email</t>
+          <t>Next Step</t>
         </is>
       </c>
       <c r="V3" s="10" t="inlineStr">
         <is>
-          <t>Next Step</t>
+          <t>Next Step Date</t>
         </is>
       </c>
       <c r="W3" s="10" t="inlineStr">
-        <is>
-          <t>Next Step Date</t>
-        </is>
-      </c>
-      <c r="X3" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1333,106 +1321,101 @@
       <c r="D4" s="28" t="n">
         <v>46096</v>
       </c>
-      <c r="E4" s="28" t="n">
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Analytics Manager</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="n">
+        <v>46092</v>
+      </c>
+      <c r="I4" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="K4" s="31" t="n">
+        <v>76</v>
+      </c>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="n"/>
+      <c r="N4" s="28" t="n">
         <v>46096</v>
       </c>
-      <c r="F4" s="27" t="inlineStr">
-        <is>
-          <t>Analytics Manager</t>
-        </is>
-      </c>
-      <c r="G4" s="29" t="inlineStr">
-        <is>
-          <t>San Diego</t>
-        </is>
-      </c>
-      <c r="H4" s="29" t="inlineStr">
-        <is>
-          <t>Posted</t>
-        </is>
-      </c>
-      <c r="I4" s="30" t="n">
-        <v>46092</v>
-      </c>
-      <c r="J4" s="31" t="n">
-        <v>24</v>
-      </c>
-      <c r="K4" s="29" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="L4" s="31" t="n">
-        <v>76</v>
-      </c>
-      <c r="M4" s="29" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N4" s="28" t="n"/>
-      <c r="O4" s="28" t="n">
-        <v>46096</v>
+      <c r="O4" s="32" t="n">
+        <v>130000</v>
       </c>
       <c r="P4" s="32" t="n">
-        <v>130000</v>
-      </c>
-      <c r="Q4" s="32" t="n">
         <v>160000</v>
       </c>
-      <c r="R4" s="33" t="inlineStr">
+      <c r="Q4" s="33" t="inlineStr">
         <is>
           <t>Linkedin, Indeed, etc (ctrl-k) to add JD hyperlink for AI</t>
         </is>
       </c>
-      <c r="S4" s="32" t="n">
+      <c r="R4" s="32" t="n">
         <v>190000</v>
       </c>
+      <c r="S4" s="29" t="n"/>
       <c r="T4" s="29" t="n"/>
       <c r="U4" s="29" t="n"/>
-      <c r="V4" s="29" t="n"/>
-      <c r="W4" s="34" t="n"/>
-      <c r="X4" s="29" t="n"/>
+      <c r="V4" s="34" t="n"/>
+      <c r="W4" s="29" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:X4"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M4 N5:N715">
+  <conditionalFormatting sqref="L4:L715">
     <cfRule type="containsText" priority="2" operator="containsText" dxfId="7" text="Applied">
-      <formula>NOT(ISERROR(SEARCH("Applied",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Applied",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="3" operator="containsText" dxfId="6" text="Phone Screen">
-      <formula>NOT(ISERROR(SEARCH("Phone Screen",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Phone Screen",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="4" operator="containsText" dxfId="2" text="Interview">
-      <formula>NOT(ISERROR(SEARCH("Interview",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Interview",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="5" operator="containsText" dxfId="2" text="Final Round">
-      <formula>NOT(ISERROR(SEARCH("Final Round",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Final Round",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="6" operator="containsText" dxfId="3" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("In Progress",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="7" operator="containsText" dxfId="2" text="Offer">
-      <formula>NOT(ISERROR(SEARCH("Offer",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Offer",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="8" operator="containsText" dxfId="1" text="Rejected">
-      <formula>NOT(ISERROR(SEARCH("Rejected",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Rejected",L4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="9" operator="containsText" dxfId="0" text="Withdrawn">
-      <formula>NOT(ISERROR(SEARCH("Withdrawn",M4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Withdrawn",L4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="2">
-    <dataValidation sqref="K4 M5:M715" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J715" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Full-Time,Part-Time,Contract,Internship,Remote,Hybrid,On-site"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="M4 N5:N715" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L4:L715" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Applied,Phone Screen,Interview,Final Round,In Progress,Offer,Rejected,Withdrawn"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
[B1] Add row-2 instruction banner + Resume Score header comment
- Row 2 (merged A2:W2): a short "how to log a job" instruction banner,
  print-friendly light-blue fill; leaves the P1/P2/P3 helper labels intact.
- Comment on the "Resume Score" header documenting it is reserved for the
  True ATS Score (auto-filled by the scorer; leave blank).

Closes the two deferred follow-ups on #24.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/job_tracker_template.xlsx
+++ b/templates/job_tracker_template.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="167" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -166,8 +166,14 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -228,6 +234,11 @@
         <bgColor rgb="FF0066CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -275,7 +286,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -440,6 +451,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -618,6 +632,12 @@
       <text>
         <t xml:space="preserve">Marc Alexander:
 Available in Linkedin (might require Premium).  I try to apply 1st day the opportunity posts and be in the 1st 100 applications. </t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>Marc Alexander:
+Reserved for the True ATS Score — written automatically by the ATS scorer (scripts/ats_score_&lt;date&gt;.py). Leave this blank; do not type a score here. A strong fit lands in the high-80s/90s; a flat 100 means the keyword list was too soft.</t>
       </text>
     </comment>
     <comment ref="M3" authorId="0" shapeId="0">
@@ -1148,30 +1168,12 @@
         </is>
       </c>
     </row>
-    <row r="2" hidden="1" ht="27.75" customHeight="1" s="42">
-      <c r="A2" s="40" t="n"/>
-      <c r="B2" s="40" t="n"/>
-      <c r="C2" s="40" t="n"/>
-      <c r="D2" s="40" t="n"/>
-      <c r="E2" s="40" t="n"/>
-      <c r="F2" s="40" t="n"/>
-      <c r="G2" s="40" t="n"/>
-      <c r="H2" s="40" t="n"/>
-      <c r="I2" s="40" t="n"/>
-      <c r="J2" s="40" t="n"/>
-      <c r="K2" s="40" t="n"/>
-      <c r="L2" s="40" t="n"/>
-      <c r="M2" s="40" t="n"/>
-      <c r="N2" s="40" t="n"/>
-      <c r="O2" s="40" t="n"/>
-      <c r="P2" s="40" t="n"/>
-      <c r="Q2" s="40" t="n"/>
-      <c r="R2" s="40" t="n"/>
-      <c r="S2" s="40" t="n"/>
-      <c r="T2" s="40" t="n"/>
-      <c r="U2" s="40" t="n"/>
-      <c r="V2" s="40" t="n"/>
-      <c r="W2" s="40" t="n"/>
+    <row r="2" hidden="1" ht="30" customHeight="1" s="42">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>How to log a job:  add one row per posting starting at row 4 — fill Company, Role / Title and Date Found, and paste the posting link in “Sourced From (w/link)”.  Status and Job Type are dropdowns.  Leave “Resume Score” blank — the ATS scorer fills it.</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>P1 Score</t>
@@ -1381,7 +1383,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:X4"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A2:W2"/>
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <conditionalFormatting sqref="L4:L715">

</xml_diff>